<commit_message>
Auto: Update market data
</commit_message>
<xml_diff>
--- a/holdings_snapshot/SMH/SMH_holdings_2026-10-12.xlsx
+++ b/holdings_snapshot/SMH/SMH_holdings_2026-10-12.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SMH_asof_20261008" sheetId="1" r:id="R7002d5c3afcf437b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SMH_asof_20261009" sheetId="1" r:id="R2653f2d2a1cd4d1a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -10,7 +10,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="174">
   <x:si>
-    <x:t>Daily Holdings (%)  10/08/2026</x:t>
+    <x:t>Daily Holdings (%)  10/09/2026</x:t>
   </x:si>
   <x:si>
     <x:t/>
@@ -52,13 +52,13 @@
     <x:t>BBG000BBJQV0</x:t>
   </x:si>
   <x:si>
-    <x:t>62,256,101</x:t>
+    <x:t>62,152,997</x:t>
   </x:si>
   <x:si>
     <x:t>Stock</x:t>
   </x:si>
   <x:si>
-    <x:t>$14,348,786,158.48</x:t>
+    <x:t>$14,250,439,152.16</x:t>
   </x:si>
   <x:si>
     <x:t> -- </x:t>
@@ -76,13 +76,13 @@
     <x:t>BBG000BD8ZK0</x:t>
   </x:si>
   <x:si>
-    <x:t>14,875,961</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$6,813,041,378.39</x:t>
-  </x:si>
-  <x:si>
-    <x:t>9.30%</x:t>
+    <x:t>14,851,325</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$6,732,254,135.75</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9.26%</x:t>
   </x:si>
   <x:si>
     <x:t>AMD</x:t>
@@ -94,13 +94,13 @@
     <x:t>BBG000BBQCY0</x:t>
   </x:si>
   <x:si>
-    <x:t>6,680,556</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$4,146,487,498.08</x:t>
-  </x:si>
-  <x:si>
-    <x:t>5.66%</x:t>
+    <x:t>6,669,492</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$4,055,718,085.20</x:t>
+  </x:si>
+  <x:si>
+    <x:t>5.58%</x:t>
   </x:si>
   <x:si>
     <x:t>AVGO</x:t>
@@ -112,13 +112,13 @@
     <x:t>BBG00KHY5S69</x:t>
   </x:si>
   <x:si>
-    <x:t>10,861,896</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$3,911,803,225.44</x:t>
-  </x:si>
-  <x:si>
-    <x:t>5.34%</x:t>
+    <x:t>10,843,864</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$3,920,490,590.56</x:t>
+  </x:si>
+  <x:si>
+    <x:t>5.39%</x:t>
   </x:si>
   <x:si>
     <x:t>MU</x:t>
@@ -130,15 +130,33 @@
     <x:t>BBG000C5Z1S3</x:t>
   </x:si>
   <x:si>
-    <x:t>3,387,172</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$3,508,568,244.48</x:t>
+    <x:t>3,381,564</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$3,479,629,356.00</x:t>
   </x:si>
   <x:si>
     <x:t>4.79%</x:t>
   </x:si>
   <x:si>
+    <x:t>MRVL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Marvell Technology Inc</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BBG00ZXBJ153</x:t>
+  </x:si>
+  <x:si>
+    <x:t>12,400,061</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$3,413,488,792.08</x:t>
+  </x:si>
+  <x:si>
+    <x:t>4.70%</x:t>
+  </x:si>
+  <x:si>
     <x:t>TXN</x:t>
   </x:si>
   <x:si>
@@ -148,28 +166,10 @@
     <x:t>BBG000BVV7G1</x:t>
   </x:si>
   <x:si>
-    <x:t>11,948,808</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$3,443,646,465.60</x:t>
-  </x:si>
-  <x:si>
-    <x:t>4.70%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MRVL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Marvell Technology Inc</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BBG00ZXBJ153</x:t>
-  </x:si>
-  <x:si>
-    <x:t>12,420,629</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$3,410,704,723.40</x:t>
+    <x:t>11,928,972</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$3,384,726,515.28</x:t>
   </x:si>
   <x:si>
     <x:t>4.66%</x:t>
@@ -184,10 +184,10 @@
     <x:t>BBG000BBPFB9</x:t>
   </x:si>
   <x:si>
-    <x:t>6,666,717</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$3,397,158,981.69</x:t>
+    <x:t>6,655,649</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$3,374,613,712.47</x:t>
   </x:si>
   <x:si>
     <x:t>4.64%</x:t>
@@ -202,10 +202,10 @@
     <x:t>BBG000BMTFR4</x:t>
   </x:si>
   <x:si>
-    <x:t>17,088,710</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$3,361,691,031.20</x:t>
+    <x:t>17,060,342</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$3,336,491,084.94</x:t>
   </x:si>
   <x:si>
     <x:t>4.59%</x:t>
@@ -220,13 +220,13 @@
     <x:t>BBG000K6MRN4</x:t>
   </x:si>
   <x:si>
-    <x:t>1,811,529</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$3,206,025,908.91</x:t>
-  </x:si>
-  <x:si>
-    <x:t>4.38%</x:t>
+    <x:t>1,808,529</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$3,219,796,519.86</x:t>
+  </x:si>
+  <x:si>
+    <x:t>4.43%</x:t>
   </x:si>
   <x:si>
     <x:t>LRCX</x:t>
@@ -238,10 +238,10 @@
     <x:t>BBG000BNFLM9</x:t>
   </x:si>
   <x:si>
-    <x:t>9,896,465</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$3,172,707,714.35</x:t>
+    <x:t>9,880,037</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$3,150,150,997.08</x:t>
   </x:si>
   <x:si>
     <x:t>4.33%</x:t>
@@ -256,13 +256,13 @@
     <x:t>BBG000C0G1D1</x:t>
   </x:si>
   <x:si>
-    <x:t>29,421,030</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$3,150,403,892.40</x:t>
-  </x:si>
-  <x:si>
-    <x:t>4.30%</x:t>
+    <x:t>29,372,190</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$3,075,268,293.00</x:t>
+  </x:si>
+  <x:si>
+    <x:t>4.23%</x:t>
   </x:si>
   <x:si>
     <x:t>ADI</x:t>
@@ -274,13 +274,13 @@
     <x:t>BBG000BB6G37</x:t>
   </x:si>
   <x:si>
-    <x:t>7,495,056</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$3,042,468,082.08</x:t>
-  </x:si>
-  <x:si>
-    <x:t>4.15%</x:t>
+    <x:t>7,482,616</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$3,039,363,793.04</x:t>
+  </x:si>
+  <x:si>
+    <x:t>4.18%</x:t>
   </x:si>
   <x:si>
     <x:t>SKHY</x:t>
@@ -292,13 +292,13 @@
     <x:t>BBG0238L5JS9</x:t>
   </x:si>
   <x:si>
-    <x:t>17,526,082</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$2,988,196,981.00</x:t>
-  </x:si>
-  <x:si>
-    <x:t>4.08%</x:t>
+    <x:t>17,497,058</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$2,957,527,713.74</x:t>
+  </x:si>
+  <x:si>
+    <x:t>4.07%</x:t>
   </x:si>
   <x:si>
     <x:t>QCOM</x:t>
@@ -310,13 +310,13 @@
     <x:t>BBG000CGC1X8</x:t>
   </x:si>
   <x:si>
-    <x:t>14,837,331</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$2,611,518,629.31</x:t>
-  </x:si>
-  <x:si>
-    <x:t>3.57%</x:t>
+    <x:t>14,812,699</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$2,599,628,674.50</x:t>
+  </x:si>
+  <x:si>
+    <x:t>3.58%</x:t>
   </x:si>
   <x:si>
     <x:t>SNPS</x:t>
@@ -328,13 +328,13 @@
     <x:t>BBG000BSFRF3</x:t>
   </x:si>
   <x:si>
-    <x:t>3,000,744</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$1,493,620,326.00</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2.04%</x:t>
+    <x:t>2,995,764</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$1,527,809,682.36</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2.10%</x:t>
   </x:si>
   <x:si>
     <x:t>CDNS</x:t>
@@ -346,13 +346,13 @@
     <x:t>BBG000C13CD9</x:t>
   </x:si>
   <x:si>
-    <x:t>4,259,675</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$1,485,945,027.00</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2.03%</x:t>
+    <x:t>4,252,603</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$1,500,488,442.52</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2.06%</x:t>
   </x:si>
   <x:si>
     <x:t>TER</x:t>
@@ -364,13 +364,13 @@
     <x:t>BBG000BV4DR6</x:t>
   </x:si>
   <x:si>
-    <x:t>2,298,781</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$916,569,960.32</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1.25%</x:t>
+    <x:t>2,294,965</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$924,136,506.20</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1.27%</x:t>
   </x:si>
   <x:si>
     <x:t>MPWR</x:t>
@@ -382,13 +382,13 @@
     <x:t>BBG000C30L48</x:t>
   </x:si>
   <x:si>
-    <x:t>647,504</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$886,950,979.20</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1.21%</x:t>
+    <x:t>646,428</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$896,136,672.12</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1.23%</x:t>
   </x:si>
   <x:si>
     <x:t>ALAB</x:t>
@@ -400,13 +400,13 @@
     <x:t>BBG00TDKHW99</x:t>
   </x:si>
   <x:si>
-    <x:t>2,318,962</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$804,795,762.10</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1.10%</x:t>
+    <x:t>2,315,114</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$792,255,161.94</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1.09%</x:t>
   </x:si>
   <x:si>
     <x:t>ARM</x:t>
@@ -418,13 +418,13 @@
     <x:t>BBG01J1GXZF0</x:t>
   </x:si>
   <x:si>
-    <x:t>2,855,183</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$786,003,328.07</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1.07%</x:t>
+    <x:t>2,850,443</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$759,015,962.04</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1.04%</x:t>
   </x:si>
   <x:si>
     <x:t>NXPI</x:t>
@@ -436,13 +436,13 @@
     <x:t>BBG000BND699</x:t>
   </x:si>
   <x:si>
-    <x:t>3,133,706</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$724,105,445.42</x:t>
-  </x:si>
-  <x:si>
-    <x:t>0.99%</x:t>
+    <x:t>3,128,502</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$711,796,775.04</x:t>
+  </x:si>
+  <x:si>
+    <x:t>0.98%</x:t>
   </x:si>
   <x:si>
     <x:t>STM</x:t>
@@ -454,10 +454,10 @@
     <x:t>BBG000BD4GX2</x:t>
   </x:si>
   <x:si>
-    <x:t>12,529,108</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$660,409,282.68</x:t>
+    <x:t>12,508,308</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$651,182,514.48</x:t>
   </x:si>
   <x:si>
     <x:t>0.90%</x:t>
@@ -472,10 +472,10 @@
     <x:t>BBG000BHCP19</x:t>
   </x:si>
   <x:si>
-    <x:t>7,362,115</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$555,986,924.80</x:t>
+    <x:t>7,349,895</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$555,284,567.25</x:t>
   </x:si>
   <x:si>
     <x:t>0.76%</x:t>
@@ -490,13 +490,13 @@
     <x:t>BBG000DV7MX4</x:t>
   </x:si>
   <x:si>
-    <x:t>4,534,838</x:t>
-  </x:si>
-  <x:si>
-    <x:t>$360,111,485.58</x:t>
-  </x:si>
-  <x:si>
-    <x:t>0.49%</x:t>
+    <x:t>4,527,310</x:t>
+  </x:si>
+  <x:si>
+    <x:t>$351,002,344.30</x:t>
+  </x:si>
+  <x:si>
+    <x:t>0.48%</x:t>
   </x:si>
   <x:si>
     <x:t>-USD CASH-</x:t>
@@ -505,13 +505,13 @@
     <x:t> </x:t>
   </x:si>
   <x:si>
-    <x:t>39,132,668</x:t>
+    <x:t>39,216,955</x:t>
   </x:si>
   <x:si>
     <x:t>Cash Bal</x:t>
   </x:si>
   <x:si>
-    <x:t>$39,132,667.67</x:t>
+    <x:t>$39,216,955.08</x:t>
   </x:si>
   <x:si>
     <x:t>0.05%</x:t>
@@ -523,7 +523,7 @@
     <x:t>Cash</x:t>
   </x:si>
   <x:si>
-    <x:t>$-463,548.02</x:t>
+    <x:t>$-1,234,969.86</x:t>
   </x:si>
   <x:si>
     <x:t>-0.00%</x:t>

</xml_diff>